<commit_message>
Updated plots, finally have it working to show all groups by lineage
</commit_message>
<xml_diff>
--- a/proliferation_growth_curves/Incucyte_sheets/processed/r2_processed.xlsx
+++ b/proliferation_growth_curves/Incucyte_sheets/processed/r2_processed.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allielas/HTP_fibroblasts_mitolyso/proliferation_growth_curves/Incucyte_sheets/processed/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD7CC69C-EEF5-D140-B4B3-740B045BE478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9C4BE3-8DFB-B242-B477-BFD918164CF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Averages" sheetId="1" r:id="rId1"/>
@@ -44,12 +44,6 @@
     <t>P20 LIN2-0A-b1 (B2)</t>
   </si>
   <si>
-    <t>P13 LIN5-0B-b3 LIN3-0A-b2 (A3)</t>
-  </si>
-  <si>
-    <t>P13 LIN5-0B-b3 LIN3-0A-b2 (B3)</t>
-  </si>
-  <si>
     <t>P15 LIN4-0B-b2 (A4)</t>
   </si>
   <si>
@@ -77,9 +71,6 @@
     <t xml:space="preserve">P20 LIN2-0A-b1 </t>
   </si>
   <si>
-    <t xml:space="preserve">P13 LIN5-0B-b3 LIN3-0A-b2 </t>
-  </si>
-  <si>
     <t xml:space="preserve">P15 LIN4-0B-b2 </t>
   </si>
   <si>
@@ -87,6 +78,15 @@
   </si>
   <si>
     <t xml:space="preserve">P13 LIN5-0B-b3 </t>
+  </si>
+  <si>
+    <t>P17 LIN3-0A-b2 (A3)</t>
+  </si>
+  <si>
+    <t>P17 LIN3-0A-b2 (B3)</t>
+  </si>
+  <si>
+    <t>P17 LIN3-0A-b2</t>
   </si>
 </sst>
 </file>
@@ -476,28 +476,28 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
@@ -508,7 +508,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -558,7 +558,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>6</v>
@@ -608,7 +608,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -658,7 +658,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -708,7 +708,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>12</v>
@@ -758,7 +758,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>14</v>
@@ -808,7 +808,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8">
         <v>16</v>
@@ -858,7 +858,7 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D9">
         <v>18</v>
@@ -908,7 +908,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10">
         <v>20</v>
@@ -958,7 +958,7 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11">
         <v>22</v>
@@ -1008,7 +1008,7 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D12">
         <v>24</v>
@@ -1058,7 +1058,7 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D13">
         <v>26</v>
@@ -1108,7 +1108,7 @@
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D14">
         <v>28</v>
@@ -1158,7 +1158,7 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D15">
         <v>30</v>
@@ -1208,7 +1208,7 @@
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D16">
         <v>32</v>
@@ -1258,7 +1258,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D17">
         <v>34</v>
@@ -1308,7 +1308,7 @@
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D18">
         <v>36</v>
@@ -1358,7 +1358,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D19">
         <v>38</v>
@@ -1408,7 +1408,7 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D20">
         <v>40</v>
@@ -1458,7 +1458,7 @@
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D21">
         <v>42</v>
@@ -1508,7 +1508,7 @@
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D22">
         <v>44</v>
@@ -1558,7 +1558,7 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D23">
         <v>46</v>
@@ -1608,7 +1608,7 @@
         <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D24">
         <v>48</v>
@@ -1658,7 +1658,7 @@
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D25">
         <v>50</v>
@@ -1708,7 +1708,7 @@
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D26">
         <v>52</v>
@@ -1758,7 +1758,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D27">
         <v>54</v>
@@ -1808,7 +1808,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D28">
         <v>56</v>
@@ -1858,7 +1858,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D29">
         <v>58</v>
@@ -1908,7 +1908,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D30">
         <v>60</v>
@@ -1958,7 +1958,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D31">
         <v>62</v>
@@ -2008,7 +2008,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D32">
         <v>64</v>
@@ -2058,7 +2058,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D33">
         <v>66</v>
@@ -2108,7 +2108,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D34">
         <v>68</v>
@@ -2158,7 +2158,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D35">
         <v>70</v>
@@ -2208,7 +2208,7 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D36">
         <v>72</v>
@@ -2331,22 +2331,22 @@
         <v>2</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -2357,7 +2357,7 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D2">
         <v>4</v>
@@ -2389,7 +2389,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>6</v>
@@ -2421,7 +2421,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>8</v>
@@ -2453,7 +2453,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D5">
         <v>10</v>
@@ -2485,7 +2485,7 @@
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D6">
         <v>12</v>
@@ -2517,7 +2517,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>14</v>
@@ -2549,7 +2549,7 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8">
         <v>16</v>
@@ -2581,7 +2581,7 @@
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D9">
         <v>18</v>
@@ -2613,7 +2613,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10">
         <v>20</v>
@@ -2645,7 +2645,7 @@
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11">
         <v>22</v>
@@ -2677,7 +2677,7 @@
         <v>2</v>
       </c>
       <c r="C12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D12">
         <v>24</v>
@@ -2709,7 +2709,7 @@
         <v>2</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D13">
         <v>26</v>
@@ -2741,7 +2741,7 @@
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D14">
         <v>28</v>
@@ -2773,7 +2773,7 @@
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D15">
         <v>30</v>
@@ -2805,7 +2805,7 @@
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D16">
         <v>32</v>
@@ -2837,7 +2837,7 @@
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D17">
         <v>34</v>
@@ -2869,7 +2869,7 @@
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D18">
         <v>36</v>
@@ -2901,7 +2901,7 @@
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D19">
         <v>38</v>
@@ -2933,7 +2933,7 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D20">
         <v>40</v>
@@ -2965,7 +2965,7 @@
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D21">
         <v>42</v>
@@ -2997,7 +2997,7 @@
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D22">
         <v>44</v>
@@ -3029,7 +3029,7 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D23">
         <v>46</v>
@@ -3061,7 +3061,7 @@
         <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D24">
         <v>48</v>
@@ -3093,7 +3093,7 @@
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D25">
         <v>50</v>
@@ -3125,7 +3125,7 @@
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D26">
         <v>52</v>
@@ -3157,7 +3157,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D27">
         <v>54</v>
@@ -3189,7 +3189,7 @@
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D28">
         <v>56</v>
@@ -3221,7 +3221,7 @@
         <v>2</v>
       </c>
       <c r="C29" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D29">
         <v>58</v>
@@ -3253,7 +3253,7 @@
         <v>2</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D30">
         <v>60</v>
@@ -3285,7 +3285,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D31">
         <v>62</v>
@@ -3317,7 +3317,7 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D32">
         <v>64</v>
@@ -3349,7 +3349,7 @@
         <v>2</v>
       </c>
       <c r="C33" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D33">
         <v>66</v>
@@ -3381,7 +3381,7 @@
         <v>2</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D34">
         <v>68</v>
@@ -3413,7 +3413,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D35">
         <v>70</v>
@@ -3445,7 +3445,7 @@
         <v>2</v>
       </c>
       <c r="C36" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D36">
         <v>72</v>

</xml_diff>